<commit_message>
Add editable org allocations, private workbook demo, and executive overhead model
</commit_message>
<xml_diff>
--- a/examples/divergent-synthetic-sample.xlsx
+++ b/examples/divergent-synthetic-sample.xlsx
@@ -10,18 +10,20 @@
     <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="OrganizationalUnits" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Employees" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Compensation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budgets" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Objectives" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="KeyResults" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CompanyAllocations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Compensation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Budgets" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Objectives" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="KeyResults" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OrganizationalUnits'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Employees'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Compensation'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Budgets'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Objectives'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'KeyResults'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OrganizationalUnits'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Employees'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CompanyAllocations'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Compensation'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Budgets'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Objectives'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'KeyResults'!$A$1:$J$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="125" customWidth="1" min="1" max="1"/>
@@ -460,7 +462,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Only the example CEO name is provided by the brief; all other people, pay, relationships, and objectives are invented.</t>
+          <t>Synthetic examples use invented people and data except the named example CEO. Actual exports retain the imported records.</t>
         </is>
       </c>
     </row>
@@ -488,54 +490,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EffectiveTo and EndDate are inclusive. Compensation periods cannot overlap.</t>
+          <t>CompanyAllocations: EmployeeID and DivergentPercent (0, 25, 50, 75, 100). Set individual contributors only. Czinger gets the remainder.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Import defaults to incremental updates; omitted rows remain. Full snapshot explicitly deactivates missing employees.</t>
+          <t>Manager splits are calculated using FTE-weighted downstream contributors; they describe team composition only, not manager payroll.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>App-owned planning records are preserved. Resolve conflicts in the planning editor.</t>
+          <t>EffectiveTo and EndDate are inclusive. Compensation periods cannot overlap.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EmploymentStatus: active / leave / inactive. UnitType: company / group / department / subdepartment.</t>
+          <t>Import defaults to incremental updates; omitted rows remain. Full snapshot explicitly deactivates missing employees.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Objective Status: on-track / at-risk / off-track / complete / not-started. Direction: increase / decrease.</t>
+          <t>App-owned planning records are preserved. Resolve conflicts in the planning editor.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ApprovedEnvelope covers a unit and all descendants. DirectAllocation reserves budget for directly assigned people.</t>
+          <t>EmploymentStatus: active / leave / inactive. UnitType: company / function / group / department / team / subteam / subdepartment.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>No objective score is calculated by averaging unrelated key results.</t>
+          <t>Objective Status: on-track / at-risk / off-track / complete / not-started. Direction: increase / decrease.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>ApprovedEnvelope covers a unit and all descendants. DirectAllocation reserves budget for directly assigned people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Optional Tier: 0 company, 1 function, 2 group, 3 department, 4 team, 5+ subteam. DepartmentCode is text; duplicates are allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>No objective score is calculated by averaging unrelated key results.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>All IDs, references, dates, FTE, pay, owners, hierarchies, and intervals are validated before commit.</t>
         </is>
@@ -552,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -560,6 +583,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -588,6 +613,16 @@
           <t>OwnerEmployeeID</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>DepartmentCode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -611,6 +646,8 @@
           <t>001</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -638,6 +675,8 @@
           <t>002</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -665,6 +704,8 @@
           <t>003</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -692,6 +733,8 @@
           <t>004</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -719,6 +762,8 @@
           <t>005</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -746,6 +791,8 @@
           <t>006</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -773,6 +820,8 @@
           <t>007</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -800,6 +849,8 @@
           <t>008</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -827,6 +878,8 @@
           <t>009</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -854,6 +907,8 @@
           <t>010</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -881,9 +936,11 @@
           <t>011</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -894,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -908,6 +965,8 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -966,6 +1025,16 @@
           <t>EmploymentType</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>SourceCompany</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>FTEBasis</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1015,6 +1084,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1068,6 +1139,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1121,6 +1194,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1174,6 +1249,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1227,6 +1304,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1280,6 +1359,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1333,6 +1414,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1386,6 +1469,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1439,6 +1524,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1492,6 +1579,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1545,6 +1634,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1598,6 +1689,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1651,6 +1744,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1704,6 +1799,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1757,6 +1854,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1810,6 +1909,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1863,6 +1964,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1916,6 +2019,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1969,6 +2074,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2022,6 +2129,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2075,6 +2184,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2128,6 +2239,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2181,6 +2294,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2234,6 +2349,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2287,6 +2404,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2340,6 +2459,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2393,6 +2514,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2446,6 +2569,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2499,6 +2624,8 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2552,14 +2679,47 @@
           <t>Full time</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>EmployeeID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>DivergentPercent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3610,7 +3770,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4017,7 +4177,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4248,7 +4408,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Limit person location choices to the four requested sites
Preserve legacy imported labels until explicitly replaced, verify saved selections, and restore the workbook contract documentation.
</commit_message>
<xml_diff>
--- a/examples/divergent-synthetic-sample.xlsx
+++ b/examples/divergent-synthetic-sample.xlsx
@@ -1131,7 +1131,7 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1186,7 +1186,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1296,7 +1296,7 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1351,7 +1351,7 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1461,7 +1461,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1516,7 +1516,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1626,7 +1626,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1681,7 +1681,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1791,7 +1791,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1846,7 +1846,7 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1956,7 +1956,7 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2011,7 +2011,7 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2121,7 +2121,7 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2176,7 +2176,7 @@
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2286,7 +2286,7 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2341,7 +2341,7 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2451,7 +2451,7 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2506,7 +2506,7 @@
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2616,7 +2616,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2671,7 +2671,7 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Torrance, CA</t>
+          <t>Los Angeles - HQ</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">

</xml_diff>

<commit_message>
Add employment-based pay, open-role views, and editable organization structure
</commit_message>
<xml_diff>
--- a/examples/divergent-synthetic-sample.xlsx
+++ b/examples/divergent-synthetic-sample.xlsx
@@ -18,9 +18,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'OrganizationalUnits'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Employees'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Employees'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CompanyAllocations'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Compensation'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Compensation'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Budgets'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Objectives'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'KeyResults'!$A$1:$J$1</definedName>
@@ -476,7 +476,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pay fields are actual annual amounts at contracted FTE. Do not multiply by FTE again. Blank pay means unknown.</t>
+          <t>PayBasis: salary (annual base + annual bonus), hourly (HourlyRate x AnnualHours), monthly (MonthlyRate x 12). Blank PayBasis retains legacy annual amounts. Never multiply pay by FTE again.</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EmploymentStatus: active / leave / inactive. UnitType: company / function / group / department / team / subteam / subdepartment.</t>
+          <t>EmploymentType: FTE or Contractor; FTE ExemptionStatus: exempt or non-exempt. EmploymentStatus: active / leave / inactive / vacant / draft. UnitType: company / function / group / department / team / subteam / subdepartment.</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -967,6 +967,7 @@
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1027,10 +1028,15 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>ExemptionStatus</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>SourceCompany</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>FTEBasis</t>
         </is>
@@ -1081,11 +1087,16 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1136,11 +1147,16 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1191,11 +1207,16 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1246,11 +1267,16 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1301,11 +1327,16 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1356,11 +1387,16 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1411,11 +1447,16 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1466,11 +1507,16 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1521,11 +1567,16 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1576,11 +1627,16 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1631,11 +1687,16 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1686,11 +1747,16 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1741,11 +1807,16 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1796,11 +1867,16 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1851,11 +1927,16 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1906,11 +1987,16 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1961,11 +2047,16 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2016,11 +2107,16 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2071,11 +2167,16 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2126,11 +2227,16 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2181,11 +2287,16 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2236,11 +2347,16 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2291,11 +2407,16 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2346,11 +2467,16 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2401,11 +2527,16 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2456,11 +2587,16 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2511,11 +2647,16 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2566,11 +2707,16 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2621,11 +2767,16 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2676,14 +2827,19 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Full time</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>exempt</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1"/>
+  <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2725,7 +2881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2735,6 +2891,10 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2773,6 +2933,26 @@
           <t>AnnualEmployerCosts</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>PayBasis</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>HourlyRate</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>AnnualHours</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>MonthlyRate</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2806,6 +2986,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2839,6 +3023,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2872,6 +3060,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2905,6 +3097,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2938,6 +3134,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2971,6 +3171,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3004,6 +3208,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3037,6 +3245,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3070,6 +3282,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3103,6 +3319,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3136,6 +3356,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3169,6 +3393,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3202,6 +3430,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3235,6 +3467,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3268,6 +3504,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3301,6 +3541,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3334,6 +3578,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3367,6 +3615,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3400,6 +3652,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3433,6 +3689,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3466,6 +3726,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3499,6 +3763,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3532,6 +3800,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3565,6 +3837,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3598,6 +3874,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3631,6 +3911,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -3664,6 +3948,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3697,6 +3985,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3730,6 +4022,10 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3763,9 +4059,13 @@
           <t>25000</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Allocate subbudgets by parent percentage with cascading dollar totals
</commit_message>
<xml_diff>
--- a/examples/divergent-synthetic-sample.xlsx
+++ b/examples/divergent-synthetic-sample.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Employees'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CompanyAllocations'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Compensation'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Budgets'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Budgets'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Objectives'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'KeyResults'!$A$1:$J$1</definedName>
   </definedNames>
@@ -469,7 +469,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IDs are text. Preserve leading zeros. Dates use YYYY-MM-DD. Currency defaults to USD; annual budgets use calendar years.</t>
+          <t>IDs are text. Preserve leading zeros. Dates use YYYY-MM-DD. Currency defaults to USD; annual budgets use calendar years. Company budgets use ApprovedEnvelope dollars; child budgets use AllocationPercent of their parent. DirectPercent reserves a share for directly assigned employees.</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4085,6 +4085,8 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4118,6 +4120,16 @@
           <t>DirectAllocation</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>AllocationPercent</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DirectPercent</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4150,6 +4162,8 @@
           <t>300000</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4182,6 +4196,8 @@
           <t>300000</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4214,6 +4230,8 @@
           <t>300000</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4246,6 +4264,8 @@
           <t>300000</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -4278,6 +4298,8 @@
           <t>300000</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4310,6 +4332,8 @@
           <t>1100000</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4342,6 +4366,8 @@
           <t>850000</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4374,6 +4400,8 @@
           <t>850000</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4406,6 +4434,8 @@
           <t>850000</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4438,6 +4468,8 @@
           <t>850000</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4470,9 +4502,11 @@
           <t>850000</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4829,7 +4863,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4915,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
@@ -4933,7 +4967,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>

</xml_diff>